<commit_message>
feat: update playwright service
</commit_message>
<xml_diff>
--- a/backend/prueba.xlsx
+++ b/backend/prueba.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lizarazo\Downloads\sicetac idea web\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4FB3CBF-6100-4F32-B152-DCC7CB117088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DC62DD9-20AD-4DC0-8A3A-A0CACF25F238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{4EEA28B7-B307-4C6B-A382-3F5C4D062489}"/>
   </bookViews>
@@ -96,7 +96,7 @@
     <t>ACHUMALAKA</t>
   </si>
   <si>
-    <t>ASA</t>
+    <t>cargado</t>
   </si>
 </sst>
 </file>

</xml_diff>